<commit_message>
fix(smd): harden legacy workbook adapter fixtures
</commit_message>
<xml_diff>
--- a/smd-process-control/tests/fixtures/aoi-sample.xlsx
+++ b/smd-process-control/tests/fixtures/aoi-sample.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AOI Line" sheetId="1" r:id="R511d2fd521924347"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="aoi model" sheetId="2" r:id="R1ae9832a285c4a54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AOI Line" sheetId="1" r:id="R7efd08e5bd064438"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="aoi model" sheetId="2" r:id="R2b84eff18faf4ca2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -901,8 +901,8 @@
       <x:c r="I9" t="n">
         <x:v>97</x:v>
       </x:c>
-      <x:c r="J9" t="str">
-        <x:v>#DIV/0!</x:v>
+      <x:c r="J9" t="n">
+        <x:v>0.97</x:v>
       </x:c>
       <x:c r="K9" t="n">
         <x:v>3</x:v>

</xml_diff>